<commit_message>
add more creel data
</commit_message>
<xml_diff>
--- a/data/current_year/recreational creel/rec_creel_catch.xlsx
+++ b/data/current_year/recreational creel/rec_creel_catch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elh/coastland/skeena-salmon-inseason-updates/data/current_year/recreational creel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5462D2FE-DC1E-0246-BCAD-ADC6E8CF76F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{899D00F3-3F2A-8A4A-9965-1DB3D081DDBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16060" yWindow="500" windowWidth="27480" windowHeight="17500" xr2:uid="{BBFB4456-6F43-5346-B932-5627D07ED1E0}"/>
+    <workbookView xWindow="18340" yWindow="500" windowWidth="27480" windowHeight="17500" xr2:uid="{BBFB4456-6F43-5346-B932-5627D07ED1E0}"/>
   </bookViews>
   <sheets>
     <sheet name="catch" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2988" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3276" uniqueCount="29">
   <si>
     <t>Year</t>
   </si>
@@ -185,8 +185,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{589E571C-CAAB-C349-8385-65B84E865495}" name="Table2" displayName="Table2" ref="A1:G721" totalsRowShown="0">
-  <autoFilter ref="A1:G721" xr:uid="{589E571C-CAAB-C349-8385-65B84E865495}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{589E571C-CAAB-C349-8385-65B84E865495}" name="Table2" displayName="Table2" ref="A1:G793" totalsRowShown="0">
+  <autoFilter ref="A1:G793" xr:uid="{589E571C-CAAB-C349-8385-65B84E865495}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{DF302C14-E33D-594D-939D-71F4B94C904C}" name="Year"/>
     <tableColumn id="2" xr3:uid="{D91F91B8-AA90-6F41-BC0B-F0AC94351025}" name="Species"/>
@@ -531,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6BCD2D2-61A9-1048-A758-3229926D6FB7}">
-  <dimension ref="A1:G721"/>
+  <dimension ref="A1:G793"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
@@ -16219,6 +16219,9 @@
       <c r="F682" t="s">
         <v>9</v>
       </c>
+      <c r="G682">
+        <v>33.1</v>
+      </c>
     </row>
     <row r="683" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A683">
@@ -16239,6 +16242,9 @@
       <c r="F683" t="s">
         <v>12</v>
       </c>
+      <c r="G683">
+        <v>15.4</v>
+      </c>
     </row>
     <row r="684" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A684">
@@ -16259,6 +16265,9 @@
       <c r="F684" t="s">
         <v>9</v>
       </c>
+      <c r="G684">
+        <v>608.9</v>
+      </c>
     </row>
     <row r="685" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A685">
@@ -16279,6 +16288,9 @@
       <c r="F685" t="s">
         <v>12</v>
       </c>
+      <c r="G685">
+        <v>396.1</v>
+      </c>
     </row>
     <row r="686" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A686">
@@ -16299,6 +16311,9 @@
       <c r="F686" t="s">
         <v>9</v>
       </c>
+      <c r="G686">
+        <v>56.5</v>
+      </c>
     </row>
     <row r="687" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A687">
@@ -16319,6 +16334,9 @@
       <c r="F687" t="s">
         <v>12</v>
       </c>
+      <c r="G687">
+        <v>27.5</v>
+      </c>
     </row>
     <row r="688" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A688">
@@ -16339,8 +16357,11 @@
       <c r="F688" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="689" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G688">
+        <v>144.9</v>
+      </c>
+    </row>
+    <row r="689" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A689">
         <v>2018</v>
       </c>
@@ -16359,8 +16380,11 @@
       <c r="F689" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="690" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G689">
+        <v>117.3</v>
+      </c>
+    </row>
+    <row r="690" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A690">
         <v>2018</v>
       </c>
@@ -16379,8 +16403,11 @@
       <c r="F690" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="691" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G690">
+        <v>893.1</v>
+      </c>
+    </row>
+    <row r="691" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A691">
         <v>2018</v>
       </c>
@@ -16399,8 +16426,11 @@
       <c r="F691" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="692" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G691">
+        <v>452.4</v>
+      </c>
+    </row>
+    <row r="692" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A692">
         <v>2018</v>
       </c>
@@ -16419,8 +16449,11 @@
       <c r="F692" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="693" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G692">
+        <v>193.8</v>
+      </c>
+    </row>
+    <row r="693" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A693">
         <v>2018</v>
       </c>
@@ -16439,8 +16472,11 @@
       <c r="F693" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="694" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G693">
+        <v>90.5</v>
+      </c>
+    </row>
+    <row r="694" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A694">
         <v>2018</v>
       </c>
@@ -16459,8 +16495,11 @@
       <c r="F694" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="695" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G694">
+        <v>432.8</v>
+      </c>
+    </row>
+    <row r="695" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A695">
         <v>2018</v>
       </c>
@@ -16479,8 +16518,11 @@
       <c r="F695" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="696" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G695">
+        <v>377.2</v>
+      </c>
+    </row>
+    <row r="696" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A696">
         <v>2018</v>
       </c>
@@ -16499,8 +16541,11 @@
       <c r="F696" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="697" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G696">
+        <v>465.9</v>
+      </c>
+    </row>
+    <row r="697" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A697">
         <v>2018</v>
       </c>
@@ -16519,8 +16564,11 @@
       <c r="F697" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="698" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G697">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="698" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A698">
         <v>2018</v>
       </c>
@@ -16539,8 +16587,11 @@
       <c r="F698" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="699" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G698">
+        <v>281.3</v>
+      </c>
+    </row>
+    <row r="699" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A699">
         <v>2018</v>
       </c>
@@ -16559,8 +16610,11 @@
       <c r="F699" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="700" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G699">
+        <v>297.10000000000002</v>
+      </c>
+    </row>
+    <row r="700" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A700">
         <v>2018</v>
       </c>
@@ -16579,8 +16633,11 @@
       <c r="F700" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="701" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G700">
+        <v>594.9</v>
+      </c>
+    </row>
+    <row r="701" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A701">
         <v>2018</v>
       </c>
@@ -16599,8 +16656,11 @@
       <c r="F701" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="702" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G701">
+        <v>618.70000000000005</v>
+      </c>
+    </row>
+    <row r="702" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A702">
         <v>2018</v>
       </c>
@@ -16619,8 +16679,11 @@
       <c r="F702" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="703" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G702">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="703" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A703">
         <v>2018</v>
       </c>
@@ -16639,8 +16702,11 @@
       <c r="F703" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="704" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G703">
+        <v>363.7</v>
+      </c>
+    </row>
+    <row r="704" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A704">
         <v>2018</v>
       </c>
@@ -16659,8 +16725,11 @@
       <c r="F704" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="705" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G704">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="705" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A705">
         <v>2018</v>
       </c>
@@ -16679,8 +16748,11 @@
       <c r="F705" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="706" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G705">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="706" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A706">
         <v>2018</v>
       </c>
@@ -16699,8 +16771,11 @@
       <c r="F706" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="707" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G706">
+        <v>49.5</v>
+      </c>
+    </row>
+    <row r="707" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A707">
         <v>2018</v>
       </c>
@@ -16719,8 +16794,11 @@
       <c r="F707" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="708" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G707">
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="708" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A708">
         <v>2018</v>
       </c>
@@ -16739,8 +16817,11 @@
       <c r="F708" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="709" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G708">
+        <v>513.4</v>
+      </c>
+    </row>
+    <row r="709" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A709">
         <v>2018</v>
       </c>
@@ -16759,8 +16840,11 @@
       <c r="F709" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="710" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G709">
+        <v>168.8</v>
+      </c>
+    </row>
+    <row r="710" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A710">
         <v>2018</v>
       </c>
@@ -16779,8 +16863,11 @@
       <c r="F710" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="711" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G710">
+        <v>40.9</v>
+      </c>
+    </row>
+    <row r="711" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A711">
         <v>2018</v>
       </c>
@@ -16799,8 +16886,11 @@
       <c r="F711" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="712" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G711">
+        <v>19.899999999999999</v>
+      </c>
+    </row>
+    <row r="712" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A712">
         <v>2018</v>
       </c>
@@ -16819,8 +16909,11 @@
       <c r="F712" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="713" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G712">
+        <v>83.9</v>
+      </c>
+    </row>
+    <row r="713" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A713">
         <v>2018</v>
       </c>
@@ -16839,8 +16932,11 @@
       <c r="F713" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="714" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G713">
+        <v>42.2</v>
+      </c>
+    </row>
+    <row r="714" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A714">
         <v>2018</v>
       </c>
@@ -16859,8 +16955,11 @@
       <c r="F714" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="715" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G714">
+        <v>677.8</v>
+      </c>
+    </row>
+    <row r="715" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A715">
         <v>2018</v>
       </c>
@@ -16879,8 +16978,11 @@
       <c r="F715" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="716" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G715">
+        <v>343.4</v>
+      </c>
+    </row>
+    <row r="716" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A716">
         <v>2018</v>
       </c>
@@ -16899,8 +17001,11 @@
       <c r="F716" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="717" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G716">
+        <v>202.1</v>
+      </c>
+    </row>
+    <row r="717" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A717">
         <v>2018</v>
       </c>
@@ -16919,8 +17024,11 @@
       <c r="F717" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="718" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G717">
+        <v>178.9</v>
+      </c>
+    </row>
+    <row r="718" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A718">
         <v>2018</v>
       </c>
@@ -16939,8 +17047,11 @@
       <c r="F718" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="719" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G718">
+        <v>133.80000000000001</v>
+      </c>
+    </row>
+    <row r="719" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A719">
         <v>2018</v>
       </c>
@@ -16959,8 +17070,11 @@
       <c r="F719" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="720" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G719">
+        <v>49.3</v>
+      </c>
+    </row>
+    <row r="720" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A720">
         <v>2018</v>
       </c>
@@ -16979,8 +17093,11 @@
       <c r="F720" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="721" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G720">
+        <v>319.39999999999998</v>
+      </c>
+    </row>
+    <row r="721" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A721">
         <v>2018</v>
       </c>
@@ -16997,6 +17114,1593 @@
         <v>25</v>
       </c>
       <c r="F721" t="s">
+        <v>12</v>
+      </c>
+      <c r="G721">
+        <v>366.3</v>
+      </c>
+    </row>
+    <row r="722" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A722">
+        <v>2021</v>
+      </c>
+      <c r="B722" t="s">
+        <v>6</v>
+      </c>
+      <c r="C722" t="s">
+        <v>7</v>
+      </c>
+      <c r="D722">
+        <v>3</v>
+      </c>
+      <c r="E722" t="s">
+        <v>8</v>
+      </c>
+      <c r="F722" t="s">
+        <v>9</v>
+      </c>
+      <c r="G722">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="723" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A723">
+        <v>2021</v>
+      </c>
+      <c r="B723" t="s">
+        <v>6</v>
+      </c>
+      <c r="C723" t="s">
+        <v>7</v>
+      </c>
+      <c r="D723">
+        <v>3</v>
+      </c>
+      <c r="E723" t="s">
+        <v>8</v>
+      </c>
+      <c r="F723" t="s">
+        <v>12</v>
+      </c>
+      <c r="G723">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="724" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A724">
+        <v>2021</v>
+      </c>
+      <c r="B724" t="s">
+        <v>6</v>
+      </c>
+      <c r="C724" t="s">
+        <v>7</v>
+      </c>
+      <c r="D724">
+        <v>3</v>
+      </c>
+      <c r="E724" t="s">
+        <v>13</v>
+      </c>
+      <c r="F724" t="s">
+        <v>9</v>
+      </c>
+      <c r="G724">
+        <v>177.2</v>
+      </c>
+    </row>
+    <row r="725" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A725">
+        <v>2021</v>
+      </c>
+      <c r="B725" t="s">
+        <v>6</v>
+      </c>
+      <c r="C725" t="s">
+        <v>7</v>
+      </c>
+      <c r="D725">
+        <v>3</v>
+      </c>
+      <c r="E725" t="s">
+        <v>13</v>
+      </c>
+      <c r="F725" t="s">
+        <v>12</v>
+      </c>
+      <c r="G725">
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="726" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A726">
+        <v>2021</v>
+      </c>
+      <c r="B726" t="s">
+        <v>6</v>
+      </c>
+      <c r="C726" t="s">
+        <v>7</v>
+      </c>
+      <c r="D726">
+        <v>3</v>
+      </c>
+      <c r="E726" t="s">
+        <v>16</v>
+      </c>
+      <c r="F726" t="s">
+        <v>9</v>
+      </c>
+      <c r="G726">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="727" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A727">
+        <v>2021</v>
+      </c>
+      <c r="B727" t="s">
+        <v>6</v>
+      </c>
+      <c r="C727" t="s">
+        <v>7</v>
+      </c>
+      <c r="D727">
+        <v>3</v>
+      </c>
+      <c r="E727" t="s">
+        <v>16</v>
+      </c>
+      <c r="F727" t="s">
+        <v>12</v>
+      </c>
+      <c r="G727">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="728" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A728">
+        <v>2021</v>
+      </c>
+      <c r="B728" t="s">
+        <v>6</v>
+      </c>
+      <c r="C728" t="s">
+        <v>7</v>
+      </c>
+      <c r="D728">
+        <v>4</v>
+      </c>
+      <c r="E728" t="s">
+        <v>17</v>
+      </c>
+      <c r="F728" t="s">
+        <v>9</v>
+      </c>
+      <c r="G728">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="729" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A729">
+        <v>2021</v>
+      </c>
+      <c r="B729" t="s">
+        <v>6</v>
+      </c>
+      <c r="C729" t="s">
+        <v>7</v>
+      </c>
+      <c r="D729">
+        <v>4</v>
+      </c>
+      <c r="E729" t="s">
+        <v>17</v>
+      </c>
+      <c r="F729" t="s">
+        <v>12</v>
+      </c>
+      <c r="G729">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="730" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A730">
+        <v>2021</v>
+      </c>
+      <c r="B730" t="s">
+        <v>6</v>
+      </c>
+      <c r="C730" t="s">
+        <v>7</v>
+      </c>
+      <c r="D730">
+        <v>4</v>
+      </c>
+      <c r="E730" t="s">
+        <v>18</v>
+      </c>
+      <c r="F730" t="s">
+        <v>9</v>
+      </c>
+      <c r="G730">
+        <v>228.3</v>
+      </c>
+    </row>
+    <row r="731" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A731">
+        <v>2021</v>
+      </c>
+      <c r="B731" t="s">
+        <v>6</v>
+      </c>
+      <c r="C731" t="s">
+        <v>7</v>
+      </c>
+      <c r="D731">
+        <v>4</v>
+      </c>
+      <c r="E731" t="s">
+        <v>18</v>
+      </c>
+      <c r="F731" t="s">
+        <v>12</v>
+      </c>
+      <c r="G731">
+        <v>153.4</v>
+      </c>
+    </row>
+    <row r="732" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A732">
+        <v>2021</v>
+      </c>
+      <c r="B732" t="s">
+        <v>6</v>
+      </c>
+      <c r="C732" t="s">
+        <v>7</v>
+      </c>
+      <c r="D732">
+        <v>4</v>
+      </c>
+      <c r="E732" t="s">
+        <v>19</v>
+      </c>
+      <c r="F732" t="s">
+        <v>9</v>
+      </c>
+      <c r="G732">
+        <v>251.4</v>
+      </c>
+    </row>
+    <row r="733" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A733">
+        <v>2021</v>
+      </c>
+      <c r="B733" t="s">
+        <v>6</v>
+      </c>
+      <c r="C733" t="s">
+        <v>7</v>
+      </c>
+      <c r="D733">
+        <v>4</v>
+      </c>
+      <c r="E733" t="s">
+        <v>19</v>
+      </c>
+      <c r="F733" t="s">
+        <v>12</v>
+      </c>
+      <c r="G733">
+        <v>60.2</v>
+      </c>
+    </row>
+    <row r="734" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A734">
+        <v>2021</v>
+      </c>
+      <c r="B734" t="s">
+        <v>6</v>
+      </c>
+      <c r="C734" t="s">
+        <v>7</v>
+      </c>
+      <c r="D734">
+        <v>4</v>
+      </c>
+      <c r="E734" t="s">
+        <v>20</v>
+      </c>
+      <c r="F734" t="s">
+        <v>9</v>
+      </c>
+      <c r="G734">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="735" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A735">
+        <v>2021</v>
+      </c>
+      <c r="B735" t="s">
+        <v>6</v>
+      </c>
+      <c r="C735" t="s">
+        <v>7</v>
+      </c>
+      <c r="D735">
+        <v>4</v>
+      </c>
+      <c r="E735" t="s">
+        <v>20</v>
+      </c>
+      <c r="F735" t="s">
+        <v>12</v>
+      </c>
+      <c r="G735">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="736" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A736">
+        <v>2021</v>
+      </c>
+      <c r="B736" t="s">
+        <v>6</v>
+      </c>
+      <c r="C736" t="s">
+        <v>7</v>
+      </c>
+      <c r="D736">
+        <v>4</v>
+      </c>
+      <c r="E736" t="s">
+        <v>21</v>
+      </c>
+      <c r="F736" t="s">
+        <v>9</v>
+      </c>
+      <c r="G736">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="737" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A737">
+        <v>2021</v>
+      </c>
+      <c r="B737" t="s">
+        <v>6</v>
+      </c>
+      <c r="C737" t="s">
+        <v>7</v>
+      </c>
+      <c r="D737">
+        <v>4</v>
+      </c>
+      <c r="E737" t="s">
+        <v>21</v>
+      </c>
+      <c r="F737" t="s">
+        <v>12</v>
+      </c>
+      <c r="G737">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="738" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A738">
+        <v>2021</v>
+      </c>
+      <c r="B738" t="s">
+        <v>6</v>
+      </c>
+      <c r="C738" t="s">
+        <v>7</v>
+      </c>
+      <c r="D738">
+        <v>4</v>
+      </c>
+      <c r="E738" t="s">
+        <v>22</v>
+      </c>
+      <c r="F738" t="s">
+        <v>9</v>
+      </c>
+      <c r="G738">
+        <v>722.3</v>
+      </c>
+    </row>
+    <row r="739" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A739">
+        <v>2021</v>
+      </c>
+      <c r="B739" t="s">
+        <v>6</v>
+      </c>
+      <c r="C739" t="s">
+        <v>7</v>
+      </c>
+      <c r="D739">
+        <v>4</v>
+      </c>
+      <c r="E739" t="s">
+        <v>22</v>
+      </c>
+      <c r="F739" t="s">
+        <v>12</v>
+      </c>
+      <c r="G739">
+        <v>239.5</v>
+      </c>
+    </row>
+    <row r="740" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A740">
+        <v>2021</v>
+      </c>
+      <c r="B740" t="s">
+        <v>6</v>
+      </c>
+      <c r="C740" t="s">
+        <v>7</v>
+      </c>
+      <c r="D740">
+        <v>4</v>
+      </c>
+      <c r="E740" t="s">
+        <v>23</v>
+      </c>
+      <c r="F740" t="s">
+        <v>9</v>
+      </c>
+      <c r="G740">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="741" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A741">
+        <v>2021</v>
+      </c>
+      <c r="B741" t="s">
+        <v>6</v>
+      </c>
+      <c r="C741" t="s">
+        <v>7</v>
+      </c>
+      <c r="D741">
+        <v>4</v>
+      </c>
+      <c r="E741" t="s">
+        <v>23</v>
+      </c>
+      <c r="F741" t="s">
+        <v>12</v>
+      </c>
+      <c r="G741">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="742" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A742">
+        <v>2021</v>
+      </c>
+      <c r="B742" t="s">
+        <v>6</v>
+      </c>
+      <c r="C742" t="s">
+        <v>7</v>
+      </c>
+      <c r="D742">
+        <v>4</v>
+      </c>
+      <c r="E742" t="s">
+        <v>24</v>
+      </c>
+      <c r="F742" t="s">
+        <v>9</v>
+      </c>
+      <c r="G742">
+        <v>32.799999999999997</v>
+      </c>
+    </row>
+    <row r="743" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A743">
+        <v>2021</v>
+      </c>
+      <c r="B743" t="s">
+        <v>6</v>
+      </c>
+      <c r="C743" t="s">
+        <v>7</v>
+      </c>
+      <c r="D743">
+        <v>4</v>
+      </c>
+      <c r="E743" t="s">
+        <v>24</v>
+      </c>
+      <c r="F743" t="s">
+        <v>12</v>
+      </c>
+      <c r="G743">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="744" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A744">
+        <v>2021</v>
+      </c>
+      <c r="B744" t="s">
+        <v>6</v>
+      </c>
+      <c r="C744" t="s">
+        <v>7</v>
+      </c>
+      <c r="D744">
+        <v>4</v>
+      </c>
+      <c r="E744" t="s">
+        <v>25</v>
+      </c>
+      <c r="F744" t="s">
+        <v>9</v>
+      </c>
+      <c r="G744">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="745" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A745">
+        <v>2021</v>
+      </c>
+      <c r="B745" t="s">
+        <v>6</v>
+      </c>
+      <c r="C745" t="s">
+        <v>7</v>
+      </c>
+      <c r="D745">
+        <v>4</v>
+      </c>
+      <c r="E745" t="s">
+        <v>25</v>
+      </c>
+      <c r="F745" t="s">
+        <v>12</v>
+      </c>
+      <c r="G745">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="746" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A746">
+        <v>2021</v>
+      </c>
+      <c r="B746" t="s">
+        <v>6</v>
+      </c>
+      <c r="C746" t="s">
+        <v>11</v>
+      </c>
+      <c r="D746">
+        <v>3</v>
+      </c>
+      <c r="E746" t="s">
+        <v>8</v>
+      </c>
+      <c r="F746" t="s">
+        <v>9</v>
+      </c>
+      <c r="G746">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="747" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A747">
+        <v>2021</v>
+      </c>
+      <c r="B747" t="s">
+        <v>6</v>
+      </c>
+      <c r="C747" t="s">
+        <v>11</v>
+      </c>
+      <c r="D747">
+        <v>3</v>
+      </c>
+      <c r="E747" t="s">
+        <v>8</v>
+      </c>
+      <c r="F747" t="s">
+        <v>12</v>
+      </c>
+      <c r="G747">
+        <v>832.1</v>
+      </c>
+    </row>
+    <row r="748" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A748">
+        <v>2021</v>
+      </c>
+      <c r="B748" t="s">
+        <v>6</v>
+      </c>
+      <c r="C748" t="s">
+        <v>11</v>
+      </c>
+      <c r="D748">
+        <v>3</v>
+      </c>
+      <c r="E748" t="s">
+        <v>13</v>
+      </c>
+      <c r="F748" t="s">
+        <v>9</v>
+      </c>
+      <c r="G748">
+        <v>519.79999999999995</v>
+      </c>
+    </row>
+    <row r="749" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A749">
+        <v>2021</v>
+      </c>
+      <c r="B749" t="s">
+        <v>6</v>
+      </c>
+      <c r="C749" t="s">
+        <v>11</v>
+      </c>
+      <c r="D749">
+        <v>3</v>
+      </c>
+      <c r="E749" t="s">
+        <v>13</v>
+      </c>
+      <c r="F749" t="s">
+        <v>12</v>
+      </c>
+      <c r="G749">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="750" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A750">
+        <v>2021</v>
+      </c>
+      <c r="B750" t="s">
+        <v>6</v>
+      </c>
+      <c r="C750" t="s">
+        <v>11</v>
+      </c>
+      <c r="D750">
+        <v>3</v>
+      </c>
+      <c r="E750" t="s">
+        <v>16</v>
+      </c>
+      <c r="F750" t="s">
+        <v>9</v>
+      </c>
+      <c r="G750">
+        <v>111.2</v>
+      </c>
+    </row>
+    <row r="751" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A751">
+        <v>2021</v>
+      </c>
+      <c r="B751" t="s">
+        <v>6</v>
+      </c>
+      <c r="C751" t="s">
+        <v>11</v>
+      </c>
+      <c r="D751">
+        <v>3</v>
+      </c>
+      <c r="E751" t="s">
+        <v>16</v>
+      </c>
+      <c r="F751" t="s">
+        <v>12</v>
+      </c>
+      <c r="G751">
+        <v>87.6</v>
+      </c>
+    </row>
+    <row r="752" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A752">
+        <v>2021</v>
+      </c>
+      <c r="B752" t="s">
+        <v>6</v>
+      </c>
+      <c r="C752" t="s">
+        <v>11</v>
+      </c>
+      <c r="D752">
+        <v>4</v>
+      </c>
+      <c r="E752" t="s">
+        <v>17</v>
+      </c>
+      <c r="F752" t="s">
+        <v>9</v>
+      </c>
+      <c r="G752">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="753" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A753">
+        <v>2021</v>
+      </c>
+      <c r="B753" t="s">
+        <v>6</v>
+      </c>
+      <c r="C753" t="s">
+        <v>11</v>
+      </c>
+      <c r="D753">
+        <v>4</v>
+      </c>
+      <c r="E753" t="s">
+        <v>17</v>
+      </c>
+      <c r="F753" t="s">
+        <v>12</v>
+      </c>
+      <c r="G753">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="754" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A754">
+        <v>2021</v>
+      </c>
+      <c r="B754" t="s">
+        <v>6</v>
+      </c>
+      <c r="C754" t="s">
+        <v>11</v>
+      </c>
+      <c r="D754">
+        <v>4</v>
+      </c>
+      <c r="E754" t="s">
+        <v>18</v>
+      </c>
+      <c r="F754" t="s">
+        <v>9</v>
+      </c>
+      <c r="G754">
+        <v>114.1</v>
+      </c>
+    </row>
+    <row r="755" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A755">
+        <v>2021</v>
+      </c>
+      <c r="B755" t="s">
+        <v>6</v>
+      </c>
+      <c r="C755" t="s">
+        <v>11</v>
+      </c>
+      <c r="D755">
+        <v>4</v>
+      </c>
+      <c r="E755" t="s">
+        <v>18</v>
+      </c>
+      <c r="F755" t="s">
+        <v>12</v>
+      </c>
+      <c r="G755">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="756" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A756">
+        <v>2021</v>
+      </c>
+      <c r="B756" t="s">
+        <v>6</v>
+      </c>
+      <c r="C756" t="s">
+        <v>11</v>
+      </c>
+      <c r="D756">
+        <v>4</v>
+      </c>
+      <c r="E756" t="s">
+        <v>19</v>
+      </c>
+      <c r="F756" t="s">
+        <v>9</v>
+      </c>
+      <c r="G756">
+        <v>141.30000000000001</v>
+      </c>
+    </row>
+    <row r="757" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A757">
+        <v>2021</v>
+      </c>
+      <c r="B757" t="s">
+        <v>6</v>
+      </c>
+      <c r="C757" t="s">
+        <v>11</v>
+      </c>
+      <c r="D757">
+        <v>4</v>
+      </c>
+      <c r="E757" t="s">
+        <v>19</v>
+      </c>
+      <c r="F757" t="s">
+        <v>12</v>
+      </c>
+      <c r="G757">
+        <v>173.8</v>
+      </c>
+    </row>
+    <row r="758" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A758">
+        <v>2021</v>
+      </c>
+      <c r="B758" t="s">
+        <v>6</v>
+      </c>
+      <c r="C758" t="s">
+        <v>11</v>
+      </c>
+      <c r="D758">
+        <v>4</v>
+      </c>
+      <c r="E758" t="s">
+        <v>20</v>
+      </c>
+      <c r="F758" t="s">
+        <v>9</v>
+      </c>
+      <c r="G758">
+        <v>253.8</v>
+      </c>
+    </row>
+    <row r="759" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A759">
+        <v>2021</v>
+      </c>
+      <c r="B759" t="s">
+        <v>6</v>
+      </c>
+      <c r="C759" t="s">
+        <v>11</v>
+      </c>
+      <c r="D759">
+        <v>4</v>
+      </c>
+      <c r="E759" t="s">
+        <v>20</v>
+      </c>
+      <c r="F759" t="s">
+        <v>12</v>
+      </c>
+      <c r="G759">
+        <v>258.8</v>
+      </c>
+    </row>
+    <row r="760" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A760">
+        <v>2021</v>
+      </c>
+      <c r="B760" t="s">
+        <v>6</v>
+      </c>
+      <c r="C760" t="s">
+        <v>11</v>
+      </c>
+      <c r="D760">
+        <v>4</v>
+      </c>
+      <c r="E760" t="s">
+        <v>21</v>
+      </c>
+      <c r="F760" t="s">
+        <v>9</v>
+      </c>
+      <c r="G760">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="761" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A761">
+        <v>2021</v>
+      </c>
+      <c r="B761" t="s">
+        <v>6</v>
+      </c>
+      <c r="C761" t="s">
+        <v>11</v>
+      </c>
+      <c r="D761">
+        <v>4</v>
+      </c>
+      <c r="E761" t="s">
+        <v>21</v>
+      </c>
+      <c r="F761" t="s">
+        <v>12</v>
+      </c>
+      <c r="G761">
+        <v>9.3000000000000007</v>
+      </c>
+    </row>
+    <row r="762" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A762">
+        <v>2021</v>
+      </c>
+      <c r="B762" t="s">
+        <v>6</v>
+      </c>
+      <c r="C762" t="s">
+        <v>11</v>
+      </c>
+      <c r="D762">
+        <v>4</v>
+      </c>
+      <c r="E762" t="s">
+        <v>22</v>
+      </c>
+      <c r="F762" t="s">
+        <v>9</v>
+      </c>
+      <c r="G762">
+        <v>425.6</v>
+      </c>
+    </row>
+    <row r="763" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A763">
+        <v>2021</v>
+      </c>
+      <c r="B763" t="s">
+        <v>6</v>
+      </c>
+      <c r="C763" t="s">
+        <v>11</v>
+      </c>
+      <c r="D763">
+        <v>4</v>
+      </c>
+      <c r="E763" t="s">
+        <v>22</v>
+      </c>
+      <c r="F763" t="s">
+        <v>12</v>
+      </c>
+      <c r="G763">
+        <v>710.3</v>
+      </c>
+    </row>
+    <row r="764" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A764">
+        <v>2021</v>
+      </c>
+      <c r="B764" t="s">
+        <v>6</v>
+      </c>
+      <c r="C764" t="s">
+        <v>11</v>
+      </c>
+      <c r="D764">
+        <v>4</v>
+      </c>
+      <c r="E764" t="s">
+        <v>23</v>
+      </c>
+      <c r="F764" t="s">
+        <v>9</v>
+      </c>
+      <c r="G764">
+        <v>109.5</v>
+      </c>
+    </row>
+    <row r="765" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A765">
+        <v>2021</v>
+      </c>
+      <c r="B765" t="s">
+        <v>6</v>
+      </c>
+      <c r="C765" t="s">
+        <v>11</v>
+      </c>
+      <c r="D765">
+        <v>4</v>
+      </c>
+      <c r="E765" t="s">
+        <v>23</v>
+      </c>
+      <c r="F765" t="s">
+        <v>12</v>
+      </c>
+      <c r="G765">
+        <v>203.5</v>
+      </c>
+    </row>
+    <row r="766" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A766">
+        <v>2021</v>
+      </c>
+      <c r="B766" t="s">
+        <v>6</v>
+      </c>
+      <c r="C766" t="s">
+        <v>11</v>
+      </c>
+      <c r="D766">
+        <v>4</v>
+      </c>
+      <c r="E766" t="s">
+        <v>24</v>
+      </c>
+      <c r="F766" t="s">
+        <v>9</v>
+      </c>
+      <c r="G766">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="767" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A767">
+        <v>2021</v>
+      </c>
+      <c r="B767" t="s">
+        <v>6</v>
+      </c>
+      <c r="C767" t="s">
+        <v>11</v>
+      </c>
+      <c r="D767">
+        <v>4</v>
+      </c>
+      <c r="E767" t="s">
+        <v>24</v>
+      </c>
+      <c r="F767" t="s">
+        <v>12</v>
+      </c>
+      <c r="G767">
+        <v>160.1</v>
+      </c>
+    </row>
+    <row r="768" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A768">
+        <v>2021</v>
+      </c>
+      <c r="B768" t="s">
+        <v>6</v>
+      </c>
+      <c r="C768" t="s">
+        <v>11</v>
+      </c>
+      <c r="D768">
+        <v>4</v>
+      </c>
+      <c r="E768" t="s">
+        <v>25</v>
+      </c>
+      <c r="F768" t="s">
+        <v>9</v>
+      </c>
+      <c r="G768">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="769" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A769">
+        <v>2021</v>
+      </c>
+      <c r="B769" t="s">
+        <v>6</v>
+      </c>
+      <c r="C769" t="s">
+        <v>11</v>
+      </c>
+      <c r="D769">
+        <v>4</v>
+      </c>
+      <c r="E769" t="s">
+        <v>25</v>
+      </c>
+      <c r="F769" t="s">
+        <v>12</v>
+      </c>
+      <c r="G769">
+        <v>40.299999999999997</v>
+      </c>
+    </row>
+    <row r="770" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A770">
+        <v>2021</v>
+      </c>
+      <c r="B770" t="s">
+        <v>6</v>
+      </c>
+      <c r="C770" t="s">
+        <v>14</v>
+      </c>
+      <c r="D770">
+        <v>3</v>
+      </c>
+      <c r="E770" t="s">
+        <v>8</v>
+      </c>
+      <c r="F770" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="771" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A771">
+        <v>2021</v>
+      </c>
+      <c r="B771" t="s">
+        <v>6</v>
+      </c>
+      <c r="C771" t="s">
+        <v>14</v>
+      </c>
+      <c r="D771">
+        <v>3</v>
+      </c>
+      <c r="E771" t="s">
+        <v>8</v>
+      </c>
+      <c r="F771" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="772" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A772">
+        <v>2021</v>
+      </c>
+      <c r="B772" t="s">
+        <v>6</v>
+      </c>
+      <c r="C772" t="s">
+        <v>14</v>
+      </c>
+      <c r="D772">
+        <v>3</v>
+      </c>
+      <c r="E772" t="s">
+        <v>13</v>
+      </c>
+      <c r="F772" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="773" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A773">
+        <v>2021</v>
+      </c>
+      <c r="B773" t="s">
+        <v>6</v>
+      </c>
+      <c r="C773" t="s">
+        <v>14</v>
+      </c>
+      <c r="D773">
+        <v>3</v>
+      </c>
+      <c r="E773" t="s">
+        <v>13</v>
+      </c>
+      <c r="F773" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="774" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A774">
+        <v>2021</v>
+      </c>
+      <c r="B774" t="s">
+        <v>6</v>
+      </c>
+      <c r="C774" t="s">
+        <v>14</v>
+      </c>
+      <c r="D774">
+        <v>3</v>
+      </c>
+      <c r="E774" t="s">
+        <v>16</v>
+      </c>
+      <c r="F774" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="775" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A775">
+        <v>2021</v>
+      </c>
+      <c r="B775" t="s">
+        <v>6</v>
+      </c>
+      <c r="C775" t="s">
+        <v>14</v>
+      </c>
+      <c r="D775">
+        <v>3</v>
+      </c>
+      <c r="E775" t="s">
+        <v>16</v>
+      </c>
+      <c r="F775" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="776" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A776">
+        <v>2021</v>
+      </c>
+      <c r="B776" t="s">
+        <v>6</v>
+      </c>
+      <c r="C776" t="s">
+        <v>14</v>
+      </c>
+      <c r="D776">
+        <v>4</v>
+      </c>
+      <c r="E776" t="s">
+        <v>17</v>
+      </c>
+      <c r="F776" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="777" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A777">
+        <v>2021</v>
+      </c>
+      <c r="B777" t="s">
+        <v>6</v>
+      </c>
+      <c r="C777" t="s">
+        <v>14</v>
+      </c>
+      <c r="D777">
+        <v>4</v>
+      </c>
+      <c r="E777" t="s">
+        <v>17</v>
+      </c>
+      <c r="F777" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="778" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A778">
+        <v>2021</v>
+      </c>
+      <c r="B778" t="s">
+        <v>6</v>
+      </c>
+      <c r="C778" t="s">
+        <v>14</v>
+      </c>
+      <c r="D778">
+        <v>4</v>
+      </c>
+      <c r="E778" t="s">
+        <v>18</v>
+      </c>
+      <c r="F778" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="779" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A779">
+        <v>2021</v>
+      </c>
+      <c r="B779" t="s">
+        <v>6</v>
+      </c>
+      <c r="C779" t="s">
+        <v>14</v>
+      </c>
+      <c r="D779">
+        <v>4</v>
+      </c>
+      <c r="E779" t="s">
+        <v>18</v>
+      </c>
+      <c r="F779" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="780" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A780">
+        <v>2021</v>
+      </c>
+      <c r="B780" t="s">
+        <v>6</v>
+      </c>
+      <c r="C780" t="s">
+        <v>14</v>
+      </c>
+      <c r="D780">
+        <v>4</v>
+      </c>
+      <c r="E780" t="s">
+        <v>19</v>
+      </c>
+      <c r="F780" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="781" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A781">
+        <v>2021</v>
+      </c>
+      <c r="B781" t="s">
+        <v>6</v>
+      </c>
+      <c r="C781" t="s">
+        <v>14</v>
+      </c>
+      <c r="D781">
+        <v>4</v>
+      </c>
+      <c r="E781" t="s">
+        <v>19</v>
+      </c>
+      <c r="F781" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="782" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A782">
+        <v>2021</v>
+      </c>
+      <c r="B782" t="s">
+        <v>6</v>
+      </c>
+      <c r="C782" t="s">
+        <v>14</v>
+      </c>
+      <c r="D782">
+        <v>4</v>
+      </c>
+      <c r="E782" t="s">
+        <v>20</v>
+      </c>
+      <c r="F782" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="783" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A783">
+        <v>2021</v>
+      </c>
+      <c r="B783" t="s">
+        <v>6</v>
+      </c>
+      <c r="C783" t="s">
+        <v>14</v>
+      </c>
+      <c r="D783">
+        <v>4</v>
+      </c>
+      <c r="E783" t="s">
+        <v>20</v>
+      </c>
+      <c r="F783" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="784" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A784">
+        <v>2021</v>
+      </c>
+      <c r="B784" t="s">
+        <v>6</v>
+      </c>
+      <c r="C784" t="s">
+        <v>14</v>
+      </c>
+      <c r="D784">
+        <v>4</v>
+      </c>
+      <c r="E784" t="s">
+        <v>21</v>
+      </c>
+      <c r="F784" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="785" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A785">
+        <v>2021</v>
+      </c>
+      <c r="B785" t="s">
+        <v>6</v>
+      </c>
+      <c r="C785" t="s">
+        <v>14</v>
+      </c>
+      <c r="D785">
+        <v>4</v>
+      </c>
+      <c r="E785" t="s">
+        <v>21</v>
+      </c>
+      <c r="F785" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="786" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A786">
+        <v>2021</v>
+      </c>
+      <c r="B786" t="s">
+        <v>6</v>
+      </c>
+      <c r="C786" t="s">
+        <v>14</v>
+      </c>
+      <c r="D786">
+        <v>4</v>
+      </c>
+      <c r="E786" t="s">
+        <v>22</v>
+      </c>
+      <c r="F786" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="787" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A787">
+        <v>2021</v>
+      </c>
+      <c r="B787" t="s">
+        <v>6</v>
+      </c>
+      <c r="C787" t="s">
+        <v>14</v>
+      </c>
+      <c r="D787">
+        <v>4</v>
+      </c>
+      <c r="E787" t="s">
+        <v>22</v>
+      </c>
+      <c r="F787" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="788" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A788">
+        <v>2021</v>
+      </c>
+      <c r="B788" t="s">
+        <v>6</v>
+      </c>
+      <c r="C788" t="s">
+        <v>14</v>
+      </c>
+      <c r="D788">
+        <v>4</v>
+      </c>
+      <c r="E788" t="s">
+        <v>23</v>
+      </c>
+      <c r="F788" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="789" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A789">
+        <v>2021</v>
+      </c>
+      <c r="B789" t="s">
+        <v>6</v>
+      </c>
+      <c r="C789" t="s">
+        <v>14</v>
+      </c>
+      <c r="D789">
+        <v>4</v>
+      </c>
+      <c r="E789" t="s">
+        <v>23</v>
+      </c>
+      <c r="F789" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="790" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A790">
+        <v>2021</v>
+      </c>
+      <c r="B790" t="s">
+        <v>6</v>
+      </c>
+      <c r="C790" t="s">
+        <v>14</v>
+      </c>
+      <c r="D790">
+        <v>4</v>
+      </c>
+      <c r="E790" t="s">
+        <v>24</v>
+      </c>
+      <c r="F790" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="791" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A791">
+        <v>2021</v>
+      </c>
+      <c r="B791" t="s">
+        <v>6</v>
+      </c>
+      <c r="C791" t="s">
+        <v>14</v>
+      </c>
+      <c r="D791">
+        <v>4</v>
+      </c>
+      <c r="E791" t="s">
+        <v>24</v>
+      </c>
+      <c r="F791" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="792" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A792">
+        <v>2021</v>
+      </c>
+      <c r="B792" t="s">
+        <v>6</v>
+      </c>
+      <c r="C792" t="s">
+        <v>14</v>
+      </c>
+      <c r="D792">
+        <v>4</v>
+      </c>
+      <c r="E792" t="s">
+        <v>25</v>
+      </c>
+      <c r="F792" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="793" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A793">
+        <v>2021</v>
+      </c>
+      <c r="B793" t="s">
+        <v>6</v>
+      </c>
+      <c r="C793" t="s">
+        <v>14</v>
+      </c>
+      <c r="D793">
+        <v>4</v>
+      </c>
+      <c r="E793" t="s">
+        <v>25</v>
+      </c>
+      <c r="F793" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
write code for recreational catch estimate plots (areas 3 and 4)
</commit_message>
<xml_diff>
--- a/data/current_year/recreational creel/rec_creel_catch.xlsx
+++ b/data/current_year/recreational creel/rec_creel_catch.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elh/coastland/skeena-salmon-inseason-updates/data/current_year/recreational creel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{899D00F3-3F2A-8A4A-9965-1DB3D081DDBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C169B9-C19A-E545-9FE5-35688F6B3178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18340" yWindow="500" windowWidth="27480" windowHeight="17500" xr2:uid="{BBFB4456-6F43-5346-B932-5627D07ED1E0}"/>
+    <workbookView xWindow="15880" yWindow="940" windowWidth="28000" windowHeight="17500" activeTab="1" xr2:uid="{BBFB4456-6F43-5346-B932-5627D07ED1E0}"/>
   </bookViews>
   <sheets>
     <sheet name="catch" sheetId="1" r:id="rId1"/>
-    <sheet name="effort" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
+    <sheet name="effort" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3276" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3830" uniqueCount="29">
   <si>
     <t>Year</t>
   </si>
@@ -130,7 +131,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -144,6 +145,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -153,7 +169,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -161,12 +177,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18714,6 +18743,3145 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{732411BF-E248-DE4A-8DE0-B02EAB7FB229}">
+  <dimension ref="A1:E184"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2017</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2">
+        <v>5229</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2017</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2017</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4">
+        <v>3800</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2017</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5">
+        <v>1811</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2017</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>2017</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>2017</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8">
+        <v>1839</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>2017</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>2017</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10">
+        <v>22871</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>2017</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11">
+        <v>3340</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>2017</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12">
+        <v>14004</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>2017</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>2017</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14">
+        <v>4632</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>2017</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15">
+        <v>3072</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>2017</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16">
+        <v>6563</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>2017</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17">
+        <v>3425</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>2017</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18">
+        <v>3410</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>2017</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>2018</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>2018</v>
+      </c>
+      <c r="B21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21">
+        <v>2121</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>2018</v>
+      </c>
+      <c r="B22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22">
+        <v>2964</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>2018</v>
+      </c>
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23">
+        <v>2612</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>2018</v>
+      </c>
+      <c r="B24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24">
+        <v>1593</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>2018</v>
+      </c>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>2018</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>2018</v>
+      </c>
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>2018</v>
+      </c>
+      <c r="B28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28">
+        <v>5758</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>2018</v>
+      </c>
+      <c r="B29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>2018</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30">
+        <v>4580</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>2018</v>
+      </c>
+      <c r="B31" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>2018</v>
+      </c>
+      <c r="B32" t="s">
+        <v>28</v>
+      </c>
+      <c r="C32" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32">
+        <v>3407</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>2018</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>2018</v>
+      </c>
+      <c r="B34" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34">
+        <v>4263</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>2018</v>
+      </c>
+      <c r="B35" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35">
+        <v>3390</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>2018</v>
+      </c>
+      <c r="B36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" t="s">
+        <v>15</v>
+      </c>
+      <c r="D36" t="s">
+        <v>9</v>
+      </c>
+      <c r="E36">
+        <v>3183</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>2018</v>
+      </c>
+      <c r="B37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37">
+        <v>2457</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>2019</v>
+      </c>
+      <c r="B38" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" t="s">
+        <v>9</v>
+      </c>
+      <c r="E38">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>2019</v>
+      </c>
+      <c r="B39" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>2019</v>
+      </c>
+      <c r="B40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40">
+        <v>5675</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>2019</v>
+      </c>
+      <c r="B41" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41">
+        <v>4735</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>2019</v>
+      </c>
+      <c r="B42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42">
+        <v>4806</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>2019</v>
+      </c>
+      <c r="B43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43">
+        <v>2382</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>2019</v>
+      </c>
+      <c r="B44" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" t="s">
+        <v>15</v>
+      </c>
+      <c r="D44" t="s">
+        <v>9</v>
+      </c>
+      <c r="E44">
+        <v>2437</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>2019</v>
+      </c>
+      <c r="B45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" t="s">
+        <v>15</v>
+      </c>
+      <c r="D45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45">
+        <v>2866</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>2019</v>
+      </c>
+      <c r="B46" t="s">
+        <v>27</v>
+      </c>
+      <c r="C46" t="s">
+        <v>7</v>
+      </c>
+      <c r="D46" t="s">
+        <v>9</v>
+      </c>
+      <c r="E46">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>2019</v>
+      </c>
+      <c r="B47" t="s">
+        <v>27</v>
+      </c>
+      <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>2019</v>
+      </c>
+      <c r="B48" t="s">
+        <v>27</v>
+      </c>
+      <c r="C48" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" t="s">
+        <v>9</v>
+      </c>
+      <c r="E48">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>2019</v>
+      </c>
+      <c r="B49" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E49">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>2019</v>
+      </c>
+      <c r="B50" t="s">
+        <v>27</v>
+      </c>
+      <c r="C50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D50" t="s">
+        <v>9</v>
+      </c>
+      <c r="E50">
+        <v>10341</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>2019</v>
+      </c>
+      <c r="B51" t="s">
+        <v>27</v>
+      </c>
+      <c r="C51" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>2019</v>
+      </c>
+      <c r="B52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C52" t="s">
+        <v>15</v>
+      </c>
+      <c r="D52" t="s">
+        <v>9</v>
+      </c>
+      <c r="E52">
+        <v>11974</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>2019</v>
+      </c>
+      <c r="B53" t="s">
+        <v>27</v>
+      </c>
+      <c r="C53" t="s">
+        <v>15</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>2019</v>
+      </c>
+      <c r="B54" t="s">
+        <v>28</v>
+      </c>
+      <c r="C54" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" t="s">
+        <v>9</v>
+      </c>
+      <c r="E54">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>2019</v>
+      </c>
+      <c r="B55" t="s">
+        <v>28</v>
+      </c>
+      <c r="C55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>2019</v>
+      </c>
+      <c r="B56" t="s">
+        <v>28</v>
+      </c>
+      <c r="C56" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" t="s">
+        <v>9</v>
+      </c>
+      <c r="E56">
+        <v>2698</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>2019</v>
+      </c>
+      <c r="B57" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57">
+        <v>2330</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>2019</v>
+      </c>
+      <c r="B58" t="s">
+        <v>28</v>
+      </c>
+      <c r="C58" t="s">
+        <v>14</v>
+      </c>
+      <c r="D58" t="s">
+        <v>9</v>
+      </c>
+      <c r="E58">
+        <v>3894</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>2019</v>
+      </c>
+      <c r="B59" t="s">
+        <v>28</v>
+      </c>
+      <c r="C59" t="s">
+        <v>14</v>
+      </c>
+      <c r="D59" t="s">
+        <v>12</v>
+      </c>
+      <c r="E59">
+        <v>3059</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>2019</v>
+      </c>
+      <c r="B60" t="s">
+        <v>28</v>
+      </c>
+      <c r="C60" t="s">
+        <v>15</v>
+      </c>
+      <c r="D60" t="s">
+        <v>9</v>
+      </c>
+      <c r="E60">
+        <v>3435</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>2019</v>
+      </c>
+      <c r="B61" t="s">
+        <v>28</v>
+      </c>
+      <c r="C61" t="s">
+        <v>15</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61">
+        <v>1769</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>2021</v>
+      </c>
+      <c r="B62" t="s">
+        <v>6</v>
+      </c>
+      <c r="C62" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" t="s">
+        <v>9</v>
+      </c>
+      <c r="E62">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>2021</v>
+      </c>
+      <c r="B63" t="s">
+        <v>6</v>
+      </c>
+      <c r="C63" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>2021</v>
+      </c>
+      <c r="B64" t="s">
+        <v>6</v>
+      </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" t="s">
+        <v>9</v>
+      </c>
+      <c r="E64">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>2021</v>
+      </c>
+      <c r="B65" t="s">
+        <v>6</v>
+      </c>
+      <c r="C65" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" t="s">
+        <v>12</v>
+      </c>
+      <c r="E65">
+        <v>3652</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>2021</v>
+      </c>
+      <c r="B66" t="s">
+        <v>6</v>
+      </c>
+      <c r="C66" t="s">
+        <v>14</v>
+      </c>
+      <c r="D66" t="s">
+        <v>9</v>
+      </c>
+      <c r="E66">
+        <v>2797</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>2021</v>
+      </c>
+      <c r="B67" t="s">
+        <v>6</v>
+      </c>
+      <c r="C67" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67">
+        <v>3694</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>2021</v>
+      </c>
+      <c r="B68" t="s">
+        <v>6</v>
+      </c>
+      <c r="C68" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68" t="s">
+        <v>9</v>
+      </c>
+      <c r="E68">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>2021</v>
+      </c>
+      <c r="B69" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" t="s">
+        <v>15</v>
+      </c>
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69">
+        <v>1799</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>2021</v>
+      </c>
+      <c r="B70" t="s">
+        <v>27</v>
+      </c>
+      <c r="C70" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70" t="s">
+        <v>9</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>2021</v>
+      </c>
+      <c r="B71" t="s">
+        <v>27</v>
+      </c>
+      <c r="C71" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" t="s">
+        <v>12</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>2021</v>
+      </c>
+      <c r="B72" t="s">
+        <v>27</v>
+      </c>
+      <c r="C72" t="s">
+        <v>11</v>
+      </c>
+      <c r="D72" t="s">
+        <v>9</v>
+      </c>
+      <c r="E72">
+        <v>3038</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>2021</v>
+      </c>
+      <c r="B73" t="s">
+        <v>27</v>
+      </c>
+      <c r="C73" t="s">
+        <v>11</v>
+      </c>
+      <c r="D73" t="s">
+        <v>12</v>
+      </c>
+      <c r="E73">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>2021</v>
+      </c>
+      <c r="B74" t="s">
+        <v>27</v>
+      </c>
+      <c r="C74" t="s">
+        <v>14</v>
+      </c>
+      <c r="D74" t="s">
+        <v>9</v>
+      </c>
+      <c r="E74">
+        <v>17685</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>2021</v>
+      </c>
+      <c r="B75" t="s">
+        <v>27</v>
+      </c>
+      <c r="C75" t="s">
+        <v>14</v>
+      </c>
+      <c r="D75" t="s">
+        <v>12</v>
+      </c>
+      <c r="E75">
+        <v>2814</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>2021</v>
+      </c>
+      <c r="B76" t="s">
+        <v>27</v>
+      </c>
+      <c r="C76" t="s">
+        <v>15</v>
+      </c>
+      <c r="D76" t="s">
+        <v>9</v>
+      </c>
+      <c r="E76">
+        <v>17403</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>2021</v>
+      </c>
+      <c r="B77" t="s">
+        <v>27</v>
+      </c>
+      <c r="C77" t="s">
+        <v>15</v>
+      </c>
+      <c r="D77" t="s">
+        <v>12</v>
+      </c>
+      <c r="E77">
+        <v>3038</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>2021</v>
+      </c>
+      <c r="B78" t="s">
+        <v>28</v>
+      </c>
+      <c r="C78" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" t="s">
+        <v>9</v>
+      </c>
+      <c r="E78">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>2021</v>
+      </c>
+      <c r="B79" t="s">
+        <v>28</v>
+      </c>
+      <c r="C79" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79" t="s">
+        <v>12</v>
+      </c>
+      <c r="E79">
+        <v>1197</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>2021</v>
+      </c>
+      <c r="B80" t="s">
+        <v>28</v>
+      </c>
+      <c r="C80" t="s">
+        <v>11</v>
+      </c>
+      <c r="D80" t="s">
+        <v>9</v>
+      </c>
+      <c r="E80">
+        <v>3725</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>2021</v>
+      </c>
+      <c r="B81" t="s">
+        <v>28</v>
+      </c>
+      <c r="C81" t="s">
+        <v>11</v>
+      </c>
+      <c r="D81" t="s">
+        <v>12</v>
+      </c>
+      <c r="E81">
+        <v>1562</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>2021</v>
+      </c>
+      <c r="B82" t="s">
+        <v>28</v>
+      </c>
+      <c r="C82" t="s">
+        <v>14</v>
+      </c>
+      <c r="D82" t="s">
+        <v>9</v>
+      </c>
+      <c r="E82">
+        <v>6518</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>2021</v>
+      </c>
+      <c r="B83" t="s">
+        <v>28</v>
+      </c>
+      <c r="C83" t="s">
+        <v>14</v>
+      </c>
+      <c r="D83" t="s">
+        <v>12</v>
+      </c>
+      <c r="E83">
+        <v>3188</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>2021</v>
+      </c>
+      <c r="B84" t="s">
+        <v>28</v>
+      </c>
+      <c r="C84" t="s">
+        <v>15</v>
+      </c>
+      <c r="D84" t="s">
+        <v>9</v>
+      </c>
+      <c r="E84">
+        <v>4929</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>2021</v>
+      </c>
+      <c r="B85" t="s">
+        <v>28</v>
+      </c>
+      <c r="C85" t="s">
+        <v>15</v>
+      </c>
+      <c r="D85" t="s">
+        <v>12</v>
+      </c>
+      <c r="E85">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>2022</v>
+      </c>
+      <c r="B86" t="s">
+        <v>6</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E86">
+        <v>1428</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>2022</v>
+      </c>
+      <c r="B87" t="s">
+        <v>6</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E87">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>2022</v>
+      </c>
+      <c r="B88" t="s">
+        <v>6</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E88">
+        <v>1564</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>2022</v>
+      </c>
+      <c r="B89" t="s">
+        <v>6</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E89">
+        <v>2297</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>2022</v>
+      </c>
+      <c r="B90" t="s">
+        <v>6</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E90">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>2022</v>
+      </c>
+      <c r="B91" t="s">
+        <v>6</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E91">
+        <v>6213</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>2022</v>
+      </c>
+      <c r="B92" t="s">
+        <v>6</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E92">
+        <v>1431</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <v>2022</v>
+      </c>
+      <c r="B93" t="s">
+        <v>6</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E93">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <v>2022</v>
+      </c>
+      <c r="B94" t="s">
+        <v>27</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E94">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>2022</v>
+      </c>
+      <c r="B95" t="s">
+        <v>27</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E95">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>2022</v>
+      </c>
+      <c r="B96" t="s">
+        <v>27</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E96">
+        <v>1356</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>2022</v>
+      </c>
+      <c r="B97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E97">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>2022</v>
+      </c>
+      <c r="B98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E98">
+        <v>13929</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>2022</v>
+      </c>
+      <c r="B99" t="s">
+        <v>27</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E99">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <v>2022</v>
+      </c>
+      <c r="B100" t="s">
+        <v>27</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E100">
+        <v>16331</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <v>2022</v>
+      </c>
+      <c r="B101" t="s">
+        <v>27</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E101">
+        <v>2423</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A102">
+        <v>2022</v>
+      </c>
+      <c r="B102" t="s">
+        <v>28</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E102">
+        <v>1385</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <v>2022</v>
+      </c>
+      <c r="B103" t="s">
+        <v>28</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E103">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <v>2022</v>
+      </c>
+      <c r="B104" t="s">
+        <v>28</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E104">
+        <v>4229</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <v>2022</v>
+      </c>
+      <c r="B105" t="s">
+        <v>28</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E105">
+        <v>2701</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A106">
+        <v>2022</v>
+      </c>
+      <c r="B106" t="s">
+        <v>28</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E106">
+        <v>5558</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A107">
+        <v>2022</v>
+      </c>
+      <c r="B107" t="s">
+        <v>28</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E107">
+        <v>2875</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A108">
+        <v>2022</v>
+      </c>
+      <c r="B108" t="s">
+        <v>28</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E108">
+        <v>3953</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A109">
+        <v>2022</v>
+      </c>
+      <c r="B109" t="s">
+        <v>28</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E109">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A110">
+        <v>2023</v>
+      </c>
+      <c r="B110" t="s">
+        <v>6</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E110">
+        <v>1191</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A111">
+        <v>2023</v>
+      </c>
+      <c r="B111" t="s">
+        <v>6</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E111">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A112">
+        <v>2023</v>
+      </c>
+      <c r="B112" t="s">
+        <v>6</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E112">
+        <v>3180</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A113">
+        <v>2023</v>
+      </c>
+      <c r="B113" t="s">
+        <v>6</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E113">
+        <v>3790</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <v>2023</v>
+      </c>
+      <c r="B114" t="s">
+        <v>6</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E114">
+        <v>1155</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <v>2023</v>
+      </c>
+      <c r="B115" t="s">
+        <v>6</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E115">
+        <v>3415</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <v>2023</v>
+      </c>
+      <c r="B116" t="s">
+        <v>6</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E116">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A117">
+        <v>2023</v>
+      </c>
+      <c r="B117" t="s">
+        <v>6</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E117">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A118">
+        <v>2023</v>
+      </c>
+      <c r="B118" t="s">
+        <v>27</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E118">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A119">
+        <v>2023</v>
+      </c>
+      <c r="B119" t="s">
+        <v>27</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E119">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A120">
+        <v>2023</v>
+      </c>
+      <c r="B120" t="s">
+        <v>27</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E120">
+        <v>2555</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A121">
+        <v>2023</v>
+      </c>
+      <c r="B121" t="s">
+        <v>27</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E121">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A122">
+        <v>2023</v>
+      </c>
+      <c r="B122" t="s">
+        <v>27</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E122">
+        <v>17360</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A123">
+        <v>2023</v>
+      </c>
+      <c r="B123" t="s">
+        <v>27</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E123">
+        <v>3800</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A124">
+        <v>2023</v>
+      </c>
+      <c r="B124" t="s">
+        <v>27</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E124">
+        <v>22608</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A125">
+        <v>2023</v>
+      </c>
+      <c r="B125" t="s">
+        <v>27</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E125">
+        <v>5470</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A126">
+        <v>2023</v>
+      </c>
+      <c r="B126" t="s">
+        <v>28</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E126">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A127">
+        <v>2023</v>
+      </c>
+      <c r="B127" t="s">
+        <v>28</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E127">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A128">
+        <v>2023</v>
+      </c>
+      <c r="B128" t="s">
+        <v>28</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E128">
+        <v>2636</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A129">
+        <v>2023</v>
+      </c>
+      <c r="B129" t="s">
+        <v>28</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E129">
+        <v>1617</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A130">
+        <v>2023</v>
+      </c>
+      <c r="B130" t="s">
+        <v>28</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E130">
+        <v>4887</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A131">
+        <v>2023</v>
+      </c>
+      <c r="B131" t="s">
+        <v>28</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E131">
+        <v>1926</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A132">
+        <v>2023</v>
+      </c>
+      <c r="B132" t="s">
+        <v>28</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E132">
+        <v>5049</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A133">
+        <v>2023</v>
+      </c>
+      <c r="B133" t="s">
+        <v>28</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E133">
+        <v>1763</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A134">
+        <v>2024</v>
+      </c>
+      <c r="B134" t="s">
+        <v>6</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E134">
+        <v>2594</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A135">
+        <v>2024</v>
+      </c>
+      <c r="B135" t="s">
+        <v>6</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E135">
+        <v>1357</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A136">
+        <v>2024</v>
+      </c>
+      <c r="B136" t="s">
+        <v>6</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E136">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A137">
+        <v>2024</v>
+      </c>
+      <c r="B137" t="s">
+        <v>6</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E137">
+        <v>4303</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A138">
+        <v>2024</v>
+      </c>
+      <c r="B138" t="s">
+        <v>6</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E138">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A139">
+        <v>2024</v>
+      </c>
+      <c r="B139" t="s">
+        <v>6</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E139">
+        <v>3433</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A140">
+        <v>2024</v>
+      </c>
+      <c r="B140" t="s">
+        <v>6</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E140">
+        <v>2525</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A141">
+        <v>2024</v>
+      </c>
+      <c r="B141" t="s">
+        <v>6</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E141">
+        <v>1511</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A142">
+        <v>2024</v>
+      </c>
+      <c r="B142" t="s">
+        <v>27</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E142">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A143">
+        <v>2024</v>
+      </c>
+      <c r="B143" t="s">
+        <v>27</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E143">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A144">
+        <v>2024</v>
+      </c>
+      <c r="B144" t="s">
+        <v>27</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E144">
+        <v>2808</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A145">
+        <v>2024</v>
+      </c>
+      <c r="B145" t="s">
+        <v>27</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E145">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A146">
+        <v>2024</v>
+      </c>
+      <c r="B146" t="s">
+        <v>27</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E146">
+        <v>15643</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A147">
+        <v>2024</v>
+      </c>
+      <c r="B147" t="s">
+        <v>27</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E147">
+        <v>1582</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A148">
+        <v>2024</v>
+      </c>
+      <c r="B148" t="s">
+        <v>27</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E148">
+        <v>10775</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A149">
+        <v>2024</v>
+      </c>
+      <c r="B149" t="s">
+        <v>27</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E149">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A150">
+        <v>2024</v>
+      </c>
+      <c r="B150" t="s">
+        <v>28</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E150">
+        <v>1795</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A151">
+        <v>2024</v>
+      </c>
+      <c r="B151" t="s">
+        <v>28</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E151">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A152">
+        <v>2024</v>
+      </c>
+      <c r="B152" t="s">
+        <v>28</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E152">
+        <v>3375</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A153">
+        <v>2024</v>
+      </c>
+      <c r="B153" t="s">
+        <v>28</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E153">
+        <v>2359</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A154">
+        <v>2024</v>
+      </c>
+      <c r="B154" t="s">
+        <v>28</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E154">
+        <v>4385</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A155">
+        <v>2024</v>
+      </c>
+      <c r="B155" t="s">
+        <v>28</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E155">
+        <v>3234</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A156">
+        <v>2024</v>
+      </c>
+      <c r="B156" t="s">
+        <v>28</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E156">
+        <v>5402</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A157">
+        <v>2024</v>
+      </c>
+      <c r="B157" t="s">
+        <v>28</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E157">
+        <v>3379</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A158">
+        <v>2025</v>
+      </c>
+      <c r="B158" t="s">
+        <v>6</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E158">
+        <v>1231</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A159">
+        <v>2025</v>
+      </c>
+      <c r="B159" t="s">
+        <v>6</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E159">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A160">
+        <v>2025</v>
+      </c>
+      <c r="B160" t="s">
+        <v>6</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E160">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A161">
+        <v>2025</v>
+      </c>
+      <c r="B161" t="s">
+        <v>6</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E161">
+        <v>2931</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A162">
+        <v>2025</v>
+      </c>
+      <c r="B162" t="s">
+        <v>6</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E162">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A163">
+        <v>2025</v>
+      </c>
+      <c r="B163" t="s">
+        <v>6</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E163">
+        <v>5186</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A164">
+        <v>2025</v>
+      </c>
+      <c r="B164" t="s">
+        <v>6</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E164">
+        <v>3029</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A165">
+        <v>2025</v>
+      </c>
+      <c r="B165" t="s">
+        <v>6</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E165">
+        <v>2343</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A166">
+        <v>2025</v>
+      </c>
+      <c r="B166" t="s">
+        <v>27</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E166">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A167">
+        <v>2025</v>
+      </c>
+      <c r="B167" t="s">
+        <v>27</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E167">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A168">
+        <v>2025</v>
+      </c>
+      <c r="B168" t="s">
+        <v>27</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E168">
+        <v>3787</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A169">
+        <v>2025</v>
+      </c>
+      <c r="B169" t="s">
+        <v>27</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E169">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A170">
+        <v>2025</v>
+      </c>
+      <c r="B170" t="s">
+        <v>27</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E170">
+        <v>17529</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A171">
+        <v>2025</v>
+      </c>
+      <c r="B171" t="s">
+        <v>27</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E171">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A172">
+        <v>2025</v>
+      </c>
+      <c r="B172" t="s">
+        <v>27</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E172">
+        <v>16727</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A173">
+        <v>2025</v>
+      </c>
+      <c r="B173" t="s">
+        <v>27</v>
+      </c>
+      <c r="C173" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E173">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A174">
+        <v>2025</v>
+      </c>
+      <c r="B174" t="s">
+        <v>28</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E174">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A175">
+        <v>2025</v>
+      </c>
+      <c r="B175" t="s">
+        <v>28</v>
+      </c>
+      <c r="C175" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E175">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A176">
+        <v>2025</v>
+      </c>
+      <c r="B176" t="s">
+        <v>28</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E176">
+        <v>2681</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A177">
+        <v>2025</v>
+      </c>
+      <c r="B177" t="s">
+        <v>28</v>
+      </c>
+      <c r="C177" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E177">
+        <v>1774</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A178">
+        <v>2025</v>
+      </c>
+      <c r="B178" t="s">
+        <v>28</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E178">
+        <v>4330</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A179">
+        <v>2025</v>
+      </c>
+      <c r="B179" t="s">
+        <v>28</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E179">
+        <v>3536</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A180">
+        <v>2025</v>
+      </c>
+      <c r="B180" t="s">
+        <v>28</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D180" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E180">
+        <v>4157</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A181">
+        <v>2025</v>
+      </c>
+      <c r="B181" t="s">
+        <v>28</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D181" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E181">
+        <v>3526</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A182">
+        <v>2026</v>
+      </c>
+      <c r="B182" t="s">
+        <v>6</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E182">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A183">
+        <v>2026</v>
+      </c>
+      <c r="B183" t="s">
+        <v>27</v>
+      </c>
+      <c r="C183" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D183" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E183">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A184">
+        <v>2026</v>
+      </c>
+      <c r="B184" t="s">
+        <v>28</v>
+      </c>
+      <c r="C184" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D184" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E184">
+        <v>1205</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2528376-73A1-DC46-A52F-1F1C44FC6F00}">
   <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
update Area 3 and 4 Creel numbers through June
</commit_message>
<xml_diff>
--- a/data/current_year/recreational creel/rec_creel_catch.xlsx
+++ b/data/current_year/recreational creel/rec_creel_catch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elh/coastland/skeena-salmon-inseason-updates/data/current_year/recreational creel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C169B9-C19A-E545-9FE5-35688F6B3178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B6FB0A2-80F4-4D47-8B11-3B06D4F5F615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15880" yWindow="940" windowWidth="28000" windowHeight="17500" activeTab="1" xr2:uid="{BBFB4456-6F43-5346-B932-5627D07ED1E0}"/>
+    <workbookView xWindow="18080" yWindow="500" windowWidth="27960" windowHeight="17500" activeTab="1" xr2:uid="{BBFB4456-6F43-5346-B932-5627D07ED1E0}"/>
   </bookViews>
   <sheets>
     <sheet name="catch" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3830" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3839" uniqueCount="29">
   <si>
     <t>Year</t>
   </si>
@@ -18744,7 +18744,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{732411BF-E248-DE4A-8DE0-B02EAB7FB229}">
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:E187"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -21873,6 +21873,57 @@
       </c>
       <c r="E184">
         <v>1205</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A185">
+        <v>2026</v>
+      </c>
+      <c r="B185" t="s">
+        <v>6</v>
+      </c>
+      <c r="C185" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D185" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E185">
+        <v>2757</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A186">
+        <v>2026</v>
+      </c>
+      <c r="B186" t="s">
+        <v>27</v>
+      </c>
+      <c r="C186" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D186" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E186">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A187">
+        <v>2026</v>
+      </c>
+      <c r="B187" t="s">
+        <v>28</v>
+      </c>
+      <c r="C187" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D187" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E187">
+        <v>3038</v>
       </c>
     </row>
   </sheetData>

</xml_diff>